<commit_message>
Update System Design chronogram
</commit_message>
<xml_diff>
--- a/docs/0004-gant-doc.xlsx
+++ b/docs/0004-gant-doc.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28DA27CD-7002-4684-8AE7-6E7BDA3402B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F09E851-A355-48E8-9D8C-BEC0F849E51C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="415" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2598,1077 +2598,7 @@
     <cellStyle name="Warning Text" xfId="23" builtinId="11" customBuiltin="1"/>
     <cellStyle name="zTextoOculto" xfId="3" xr:uid="{26E66EE6-E33F-4D77-BAE4-0FB4F5BBF673}"/>
   </cellStyles>
-  <dxfs count="121">
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.34998626667073579"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.34998626667073579"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.34998626667073579"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.34998626667073579"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.34998626667073579"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.34998626667073579"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.34998626667073579"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.34998626667073579"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.34998626667073579"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.34998626667073579"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.34998626667073579"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.34998626667073579"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.34998626667073579"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.34998626667073579"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.34998626667073579"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.34998626667073579"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.34998626667073579"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-9.9948118533890809E-2"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.34998626667073579"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.34998626667073579"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-9.9948118533890809E-2"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="6"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="1" tint="0.34998626667073579"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left/>
-        <right/>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
+  <dxfs count="56">
     <dxf>
       <font>
         <color auto="1"/>
@@ -3951,6 +2881,110 @@
         <bottom style="thin">
           <color theme="0" tint="-0.34998626667073579"/>
         </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.34998626667073579"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="6"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.34998626667073579"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left/>
+        <right/>
+        <top/>
+        <bottom/>
       </border>
     </dxf>
     <dxf>
@@ -4337,21 +3371,21 @@
   </dxfs>
   <tableStyles count="2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="Estilo de tabela de Gantt" pivot="0" count="4" xr9:uid="{4904D139-63E4-4221-B7C9-C6C5B7A50FAF}">
-      <tableStyleElement type="wholeTable" dxfId="120"/>
-      <tableStyleElement type="headerRow" dxfId="119"/>
-      <tableStyleElement type="firstRowStripe" dxfId="118"/>
-      <tableStyleElement type="secondRowStripe" dxfId="117"/>
+      <tableStyleElement type="wholeTable" dxfId="55"/>
+      <tableStyleElement type="headerRow" dxfId="54"/>
+      <tableStyleElement type="firstRowStripe" dxfId="53"/>
+      <tableStyleElement type="secondRowStripe" dxfId="52"/>
     </tableStyle>
     <tableStyle name="ListaDeAfazeres" pivot="0" count="9" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="wholeTable" dxfId="116"/>
-      <tableStyleElement type="headerRow" dxfId="115"/>
-      <tableStyleElement type="totalRow" dxfId="114"/>
-      <tableStyleElement type="firstColumn" dxfId="113"/>
-      <tableStyleElement type="lastColumn" dxfId="112"/>
-      <tableStyleElement type="firstRowStripe" dxfId="111"/>
-      <tableStyleElement type="secondRowStripe" dxfId="110"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="109"/>
-      <tableStyleElement type="secondColumnStripe" dxfId="108"/>
+      <tableStyleElement type="wholeTable" dxfId="51"/>
+      <tableStyleElement type="headerRow" dxfId="50"/>
+      <tableStyleElement type="totalRow" dxfId="49"/>
+      <tableStyleElement type="firstColumn" dxfId="48"/>
+      <tableStyleElement type="lastColumn" dxfId="47"/>
+      <tableStyleElement type="firstRowStripe" dxfId="46"/>
+      <tableStyleElement type="secondRowStripe" dxfId="45"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="44"/>
+      <tableStyleElement type="secondColumnStripe" dxfId="43"/>
     </tableStyle>
   </tableStyles>
   <colors>
@@ -4680,7 +3714,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{0EDB95CA-98FE-4198-8801-690B9B480FDF}" name="Milestones435" displayName="Milestones435" ref="B9:H51" totalsRowShown="0" headerRowDxfId="107">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{0EDB95CA-98FE-4198-8801-690B9B480FDF}" name="Milestones435" displayName="Milestones435" ref="B9:H51" totalsRowShown="0" headerRowDxfId="42">
   <autoFilter ref="B9:H51" xr:uid="{29E5A880-80D5-4B65-B5FB-8FB3913D3D27}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -4691,11 +3725,11 @@
     <filterColumn colId="6" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{6E47A83D-ACD7-4EB6-9B84-5195E813945E}" name="TAG" dataDxfId="106"/>
-    <tableColumn id="8" xr3:uid="{D75147D4-E518-4B66-940B-B1AABBE3464D}" name="Descrição do marco" dataDxfId="105"/>
-    <tableColumn id="2" xr3:uid="{529EEF64-D037-4ACF-8CA4-0C10FE2D1FBB}" name="Categoria" dataDxfId="104"/>
-    <tableColumn id="7" xr3:uid="{23FA21E5-141F-4FE6-A103-9A25CFC820EE}" name="Tipo" dataDxfId="103"/>
-    <tableColumn id="3" xr3:uid="{711D01BA-2785-403A-9636-CCC7E2ADA584}" name="A quem?" dataDxfId="102"/>
+    <tableColumn id="1" xr3:uid="{6E47A83D-ACD7-4EB6-9B84-5195E813945E}" name="TAG" dataDxfId="41"/>
+    <tableColumn id="8" xr3:uid="{D75147D4-E518-4B66-940B-B1AABBE3464D}" name="Descrição do marco" dataDxfId="40"/>
+    <tableColumn id="2" xr3:uid="{529EEF64-D037-4ACF-8CA4-0C10FE2D1FBB}" name="Categoria" dataDxfId="39"/>
+    <tableColumn id="7" xr3:uid="{23FA21E5-141F-4FE6-A103-9A25CFC820EE}" name="Tipo" dataDxfId="38"/>
+    <tableColumn id="3" xr3:uid="{711D01BA-2785-403A-9636-CCC7E2ADA584}" name="A quem?" dataDxfId="37"/>
     <tableColumn id="5" xr3:uid="{D6D72902-F68F-4E59-A714-AFFF520C647A}" name="Início" dataCellStyle="Data"/>
     <tableColumn id="6" xr3:uid="{93E698DE-286F-49ED-AA20-D0C843671DE8}" name="Dias"/>
   </tableColumns>
@@ -4709,7 +3743,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{DD82988E-1813-40AE-BDE7-9F0200A703CB}" name="Milestones4352" displayName="Milestones4352" ref="B9:G36" totalsRowShown="0" headerRowDxfId="101" dataDxfId="100">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{DD82988E-1813-40AE-BDE7-9F0200A703CB}" name="Milestones4352" displayName="Milestones4352" ref="B9:G36" totalsRowShown="0" headerRowDxfId="36" dataDxfId="35">
   <autoFilter ref="B9:G36" xr:uid="{29E5A880-80D5-4B65-B5FB-8FB3913D3D27}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -4719,12 +3753,12 @@
     <filterColumn colId="5" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{619BF8F6-D0F1-41AD-871D-FE0240C45A93}" name="Descrição do marco" dataDxfId="99"/>
-    <tableColumn id="2" xr3:uid="{39BD914E-FB02-4352-846C-6D59624DC0B0}" name="Categoria" dataDxfId="98"/>
-    <tableColumn id="3" xr3:uid="{D274194F-BCA0-44F3-84B2-217254EE241C}" name="Atribuído a" dataDxfId="97"/>
-    <tableColumn id="4" xr3:uid="{8385BC6F-56EE-4363-A106-8DB0A1E4EF5A}" name="Progresso" dataDxfId="96"/>
-    <tableColumn id="5" xr3:uid="{02926609-7B93-4B6F-BE96-92EC7A949E4B}" name="Início" dataDxfId="95" dataCellStyle="Data"/>
-    <tableColumn id="6" xr3:uid="{8FF9BE8E-04B7-4B39-AC27-D2E534204BC3}" name="Dias" dataDxfId="94"/>
+    <tableColumn id="1" xr3:uid="{619BF8F6-D0F1-41AD-871D-FE0240C45A93}" name="Descrição do marco" dataDxfId="34"/>
+    <tableColumn id="2" xr3:uid="{39BD914E-FB02-4352-846C-6D59624DC0B0}" name="Categoria" dataDxfId="33"/>
+    <tableColumn id="3" xr3:uid="{D274194F-BCA0-44F3-84B2-217254EE241C}" name="Atribuído a" dataDxfId="32"/>
+    <tableColumn id="4" xr3:uid="{8385BC6F-56EE-4363-A106-8DB0A1E4EF5A}" name="Progresso" dataDxfId="31"/>
+    <tableColumn id="5" xr3:uid="{02926609-7B93-4B6F-BE96-92EC7A949E4B}" name="Início" dataDxfId="30" dataCellStyle="Data"/>
+    <tableColumn id="6" xr3:uid="{8FF9BE8E-04B7-4B39-AC27-D2E534204BC3}" name="Dias" dataDxfId="29"/>
   </tableColumns>
   <tableStyleInfo name="ListaDeAfazeres" showFirstColumn="1" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
   <extLst>
@@ -4736,7 +3770,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{876EA49D-634E-482B-8173-880F7B761E2C}" name="Milestones43524" displayName="Milestones43524" ref="B9:G36" totalsRowShown="0" headerRowDxfId="93">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{876EA49D-634E-482B-8173-880F7B761E2C}" name="Milestones43524" displayName="Milestones43524" ref="B9:G36" totalsRowShown="0" headerRowDxfId="28">
   <autoFilter ref="B9:G36" xr:uid="{29E5A880-80D5-4B65-B5FB-8FB3913D3D27}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -4746,9 +3780,9 @@
     <filterColumn colId="5" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{0971B905-713A-4980-8BBC-DF959C2E61F9}" name="Descrição do marco" dataDxfId="92"/>
-    <tableColumn id="2" xr3:uid="{4492A0B8-068F-4002-9E8D-E1F5FED367F0}" name="Categoria" dataDxfId="91"/>
-    <tableColumn id="3" xr3:uid="{DF1A764E-7050-4528-B7F9-B6AB99372146}" name="Atribuído a" dataDxfId="90"/>
+    <tableColumn id="1" xr3:uid="{0971B905-713A-4980-8BBC-DF959C2E61F9}" name="Descrição do marco" dataDxfId="27"/>
+    <tableColumn id="2" xr3:uid="{4492A0B8-068F-4002-9E8D-E1F5FED367F0}" name="Categoria" dataDxfId="26"/>
+    <tableColumn id="3" xr3:uid="{DF1A764E-7050-4528-B7F9-B6AB99372146}" name="Atribuído a" dataDxfId="25"/>
     <tableColumn id="4" xr3:uid="{47C54592-75B0-4C70-BBF8-0F40483670E9}" name="Progresso"/>
     <tableColumn id="5" xr3:uid="{663FB5E0-7616-4EA5-B56A-FF069E2E07D7}" name="Início" dataCellStyle="Data"/>
     <tableColumn id="6" xr3:uid="{3B766962-C06F-4E12-BE91-12AB93439874}" name="Dias"/>
@@ -6518,7 +5552,7 @@
       </c>
       <c r="I12" s="17"/>
       <c r="J12" s="40" t="str">
-        <f t="shared" ref="J12:Y50" ca="1" si="5">IF(
+        <f t="shared" ref="J12:Y31" ca="1" si="5">IF(
     AND(
         J$7&gt;=$G12,
         J$7&lt;=WORKDAY($G12,$H12-1),
@@ -6764,7 +5798,7 @@
         <v>35</v>
       </c>
       <c r="D13" s="19" t="s">
-        <v>25</v>
+        <v>122</v>
       </c>
       <c r="E13" s="19" t="s">
         <v>53</v>
@@ -6788,9 +5822,9 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-      <c r="L13" s="40" t="str">
-        <f t="shared" ca="1" si="4"/>
-        <v/>
+      <c r="L13" s="40">
+        <f t="shared" ca="1" si="4"/>
+        <v>0</v>
       </c>
       <c r="M13" s="40" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -7015,7 +6049,7 @@
         <v>36</v>
       </c>
       <c r="D14" s="19" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E14" s="19" t="s">
         <v>54</v>
@@ -7266,7 +6300,7 @@
         <v>37</v>
       </c>
       <c r="D15" s="19" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E15" s="19" t="s">
         <v>53</v>
@@ -7427,7 +6461,7 @@
         <v/>
       </c>
       <c r="AT15" s="40" t="str">
-        <f t="shared" ref="AT15:BI50" ca="1" si="6">IF(
+        <f t="shared" ref="AT15:BI30" ca="1" si="6">IF(
     AND(
         AT$7&gt;=$G15,
         AT$7&lt;=WORKDAY($G15,$H15-1),
@@ -7503,7 +6537,7 @@
         <v/>
       </c>
       <c r="BJ15" s="40" t="str">
-        <f t="shared" ref="BJ15:BM50" ca="1" si="7">IF(
+        <f t="shared" ref="BJ15:BM30" ca="1" si="7">IF(
     AND(
         BJ$7&gt;=$G15,
         BJ$7&lt;=WORKDAY($G15,$H15-1),
@@ -7541,7 +6575,7 @@
         <v>38</v>
       </c>
       <c r="D16" s="19" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E16" s="19" t="s">
         <v>54</v>
@@ -7622,7 +6656,7 @@
         <v/>
       </c>
       <c r="Z16" s="40" t="str">
-        <f t="shared" ref="Z16:AO50" ca="1" si="8">IF(
+        <f t="shared" ref="Z16:AO33" ca="1" si="8">IF(
     AND(
         Z$7&gt;=$G16,
         Z$7&lt;=WORKDAY($G16,$H16-1),
@@ -7698,7 +6732,7 @@
         <v/>
       </c>
       <c r="AP16" s="40" t="str">
-        <f t="shared" ref="AP16:BE50" ca="1" si="9">IF(
+        <f t="shared" ref="AP16:BE31" ca="1" si="9">IF(
     AND(
         AP$7&gt;=$G16,
         AP$7&lt;=WORKDAY($G16,$H16-1),
@@ -7816,7 +6850,7 @@
         <v>39</v>
       </c>
       <c r="D17" s="19" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E17" s="19" t="s">
         <v>54</v>
@@ -7844,9 +6878,9 @@
         <f t="shared" ca="1" si="5"/>
         <v/>
       </c>
-      <c r="M17" s="40">
-        <f t="shared" ca="1" si="5"/>
-        <v>2</v>
+      <c r="M17" s="40" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
       </c>
       <c r="N17" s="40" t="str">
         <f t="shared" ca="1" si="5"/>
@@ -7856,9 +6890,9 @@
         <f t="shared" ca="1" si="5"/>
         <v/>
       </c>
-      <c r="P17" s="40">
-        <f t="shared" ca="1" si="5"/>
-        <v>2</v>
+      <c r="P17" s="40" t="str">
+        <f t="shared" ca="1" si="5"/>
+        <v/>
       </c>
       <c r="Q17" s="40" t="str">
         <f t="shared" ca="1" si="5"/>
@@ -11379,7 +10413,7 @@
         <v/>
       </c>
       <c r="U31" s="40" t="str">
-        <f t="shared" ref="U31:AJ50" ca="1" si="10">IF(
+        <f t="shared" ref="U31:AJ46" ca="1" si="10">IF(
     AND(
         U$7&gt;=$G31,
         U$7&lt;=WORKDAY($G31,$H31-1),
@@ -11535,7 +10569,7 @@
         <v/>
       </c>
       <c r="BE31" s="40" t="str">
-        <f t="shared" ref="BE31:BM50" ca="1" si="11">IF(
+        <f t="shared" ref="BE31:BM49" ca="1" si="11">IF(
     AND(
         BE$7&gt;=$G31,
         BE$7&lt;=WORKDAY($G31,$H31-1),
@@ -11610,7 +10644,7 @@
       </c>
       <c r="I32" s="17"/>
       <c r="J32" s="40" t="str">
-        <f t="shared" ref="J32:Y50" ca="1" si="12">IF(
+        <f t="shared" ref="J32:Y47" ca="1" si="12">IF(
     AND(
         J$7&gt;=$G32,
         J$7&lt;=WORKDAY($G32,$H32-1),
@@ -11750,7 +10784,7 @@
         <v/>
       </c>
       <c r="AP32" s="40" t="str">
-        <f t="shared" ref="AP32:BE50" ca="1" si="13">IF(
+        <f t="shared" ref="AP32:BE49" ca="1" si="13">IF(
     AND(
         AP$7&gt;=$G32,
         AP$7&lt;=WORKDAY($G32,$H32-1),
@@ -16504,31 +15538,31 @@
   </mergeCells>
   <phoneticPr fontId="47" type="noConversion"/>
   <conditionalFormatting sqref="J6:AN6">
-    <cfRule type="expression" dxfId="13" priority="5">
+    <cfRule type="expression" dxfId="24" priority="5">
       <formula>J$7&lt;=EOMONTH($J$7,0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J6:BM6">
-    <cfRule type="expression" dxfId="12" priority="3">
+    <cfRule type="expression" dxfId="23" priority="3">
       <formula>AND(J$7&lt;=EOMONTH($J$7,1),J$7&gt;EOMONTH($J$7,0))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J11:BM50">
-    <cfRule type="expression" dxfId="11" priority="66" stopIfTrue="1">
+    <cfRule type="expression" dxfId="22" priority="66" stopIfTrue="1">
       <formula>AND($D11="Baixo risco",J$7&gt;=$G11,J$7&lt;=WORKDAY($G11,$H11-1),WEEKDAY(J$7,2)&lt;=5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="67" stopIfTrue="1">
+    <cfRule type="expression" dxfId="21" priority="67" stopIfTrue="1">
       <formula>AND($D11="Alto risco",J$7&gt;=$G11,J$7&lt;=WORKDAY($G11,$H11-1),WEEKDAY(J$7,2)&lt;=5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="68" stopIfTrue="1">
+    <cfRule type="expression" dxfId="20" priority="68" stopIfTrue="1">
       <formula>AND($D11="No prazo",J$7&gt;=$G11,J$7&lt;=WORKDAY($G11,$H11-1),WEEKDAY(J$7,2)&lt;=5)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="69" stopIfTrue="1">
+    <cfRule type="expression" dxfId="19" priority="69" stopIfTrue="1">
       <formula>AND($D11="Médio risco",J$7&gt;=$G11,J$7&lt;=WORKDAY($G11,$H11-1),WEEKDAY(J$7,2)&lt;=5)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K6:BM6">
-    <cfRule type="expression" dxfId="7" priority="4">
+    <cfRule type="expression" dxfId="18" priority="4">
       <formula>AND(K$7&lt;=EOMONTH($J$7,2),K$7&gt;EOMONTH($J$7,0),K$7&gt;EOMONTH($J$7,1))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -16783,7 +15817,7 @@
       </c>
       <c r="C6" s="71" cm="1">
         <f t="array" aca="1" ref="C6" ca="1">IFERROR(IF(MIN(Milestones4352[Início])=0,TODAY(),B11(Milestones4352[Início])),TODAY())</f>
-        <v>46177</v>
+        <v>46179</v>
       </c>
       <c r="D6" s="72"/>
       <c r="E6" s="66"/>
@@ -16886,227 +15920,227 @@
       <c r="H7" s="74"/>
       <c r="I7" s="106">
         <f ca="1">IFERROR(Início_do_projeto+Incremento_de_Rolagem,TODAY())</f>
-        <v>46178</v>
+        <v>46180</v>
       </c>
       <c r="J7" s="107">
         <f ca="1">I7+1</f>
-        <v>46179</v>
+        <v>46181</v>
       </c>
       <c r="K7" s="107">
         <f t="shared" ref="K7:AX7" ca="1" si="0">J7+1</f>
-        <v>46180</v>
+        <v>46182</v>
       </c>
       <c r="L7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46181</v>
+        <v>46183</v>
       </c>
       <c r="M7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46182</v>
+        <v>46184</v>
       </c>
       <c r="N7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46183</v>
+        <v>46185</v>
       </c>
       <c r="O7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46184</v>
+        <v>46186</v>
       </c>
       <c r="P7" s="107">
         <f ca="1">O7+1</f>
-        <v>46185</v>
+        <v>46187</v>
       </c>
       <c r="Q7" s="107">
         <f ca="1">P7+1</f>
-        <v>46186</v>
+        <v>46188</v>
       </c>
       <c r="R7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46187</v>
+        <v>46189</v>
       </c>
       <c r="S7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46188</v>
+        <v>46190</v>
       </c>
       <c r="T7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46189</v>
+        <v>46191</v>
       </c>
       <c r="U7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46190</v>
+        <v>46192</v>
       </c>
       <c r="V7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46191</v>
+        <v>46193</v>
       </c>
       <c r="W7" s="107">
         <f ca="1">V7+1</f>
-        <v>46192</v>
+        <v>46194</v>
       </c>
       <c r="X7" s="107">
         <f ca="1">W7+1</f>
-        <v>46193</v>
+        <v>46195</v>
       </c>
       <c r="Y7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46194</v>
+        <v>46196</v>
       </c>
       <c r="Z7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46195</v>
+        <v>46197</v>
       </c>
       <c r="AA7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46196</v>
+        <v>46198</v>
       </c>
       <c r="AB7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46197</v>
+        <v>46199</v>
       </c>
       <c r="AC7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46198</v>
+        <v>46200</v>
       </c>
       <c r="AD7" s="107">
         <f ca="1">AC7+1</f>
-        <v>46199</v>
+        <v>46201</v>
       </c>
       <c r="AE7" s="107">
         <f ca="1">AD7+1</f>
-        <v>46200</v>
+        <v>46202</v>
       </c>
       <c r="AF7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46201</v>
+        <v>46203</v>
       </c>
       <c r="AG7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46202</v>
+        <v>46204</v>
       </c>
       <c r="AH7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46203</v>
+        <v>46205</v>
       </c>
       <c r="AI7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46204</v>
+        <v>46206</v>
       </c>
       <c r="AJ7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46205</v>
+        <v>46207</v>
       </c>
       <c r="AK7" s="107">
         <f ca="1">AJ7+1</f>
-        <v>46206</v>
+        <v>46208</v>
       </c>
       <c r="AL7" s="107">
         <f ca="1">AK7+1</f>
-        <v>46207</v>
+        <v>46209</v>
       </c>
       <c r="AM7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46208</v>
+        <v>46210</v>
       </c>
       <c r="AN7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46209</v>
+        <v>46211</v>
       </c>
       <c r="AO7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46210</v>
+        <v>46212</v>
       </c>
       <c r="AP7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46211</v>
+        <v>46213</v>
       </c>
       <c r="AQ7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46212</v>
+        <v>46214</v>
       </c>
       <c r="AR7" s="107">
         <f ca="1">AQ7+1</f>
-        <v>46213</v>
+        <v>46215</v>
       </c>
       <c r="AS7" s="107">
         <f ca="1">AR7+1</f>
-        <v>46214</v>
+        <v>46216</v>
       </c>
       <c r="AT7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46215</v>
+        <v>46217</v>
       </c>
       <c r="AU7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46216</v>
+        <v>46218</v>
       </c>
       <c r="AV7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46217</v>
+        <v>46219</v>
       </c>
       <c r="AW7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46218</v>
+        <v>46220</v>
       </c>
       <c r="AX7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46219</v>
+        <v>46221</v>
       </c>
       <c r="AY7" s="107">
         <f ca="1">AX7+1</f>
-        <v>46220</v>
+        <v>46222</v>
       </c>
       <c r="AZ7" s="107">
         <f ca="1">AY7+1</f>
-        <v>46221</v>
+        <v>46223</v>
       </c>
       <c r="BA7" s="107">
         <f t="shared" ref="BA7:BE7" ca="1" si="1">AZ7+1</f>
-        <v>46222</v>
+        <v>46224</v>
       </c>
       <c r="BB7" s="107">
         <f t="shared" ca="1" si="1"/>
-        <v>46223</v>
+        <v>46225</v>
       </c>
       <c r="BC7" s="107">
         <f t="shared" ca="1" si="1"/>
-        <v>46224</v>
+        <v>46226</v>
       </c>
       <c r="BD7" s="107">
         <f t="shared" ca="1" si="1"/>
-        <v>46225</v>
+        <v>46227</v>
       </c>
       <c r="BE7" s="108">
         <f t="shared" ca="1" si="1"/>
-        <v>46226</v>
+        <v>46228</v>
       </c>
       <c r="BF7" s="107">
         <f ca="1">BE7+1</f>
-        <v>46227</v>
+        <v>46229</v>
       </c>
       <c r="BG7" s="107">
         <f ca="1">BF7+1</f>
-        <v>46228</v>
+        <v>46230</v>
       </c>
       <c r="BH7" s="107">
         <f t="shared" ref="BH7:BL7" ca="1" si="2">BG7+1</f>
-        <v>46229</v>
+        <v>46231</v>
       </c>
       <c r="BI7" s="107">
         <f t="shared" ca="1" si="2"/>
-        <v>46230</v>
+        <v>46232</v>
       </c>
       <c r="BJ7" s="107">
         <f t="shared" ca="1" si="2"/>
-        <v>46231</v>
+        <v>46233</v>
       </c>
       <c r="BK7" s="107">
         <f t="shared" ca="1" si="2"/>
-        <v>46232</v>
+        <v>46234</v>
       </c>
       <c r="BL7" s="108">
         <f t="shared" ca="1" si="2"/>
-        <v>46233</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="8" spans="1:68" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -17198,7 +16232,7 @@
       <c r="H9" s="79"/>
       <c r="I9" s="88" t="str">
         <f t="shared" ref="I9:BL9" ca="1" si="3">LEFT(TEXT(I7,"ddd"),1)</f>
-        <v>s</v>
+        <v>d</v>
       </c>
       <c r="J9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -17206,27 +16240,27 @@
       </c>
       <c r="K9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>t</v>
       </c>
       <c r="L9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="M9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>t</v>
+        <v>q</v>
       </c>
       <c r="N9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="O9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="P9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>d</v>
       </c>
       <c r="Q9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -17234,27 +16268,27 @@
       </c>
       <c r="R9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>t</v>
       </c>
       <c r="S9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="T9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>t</v>
+        <v>q</v>
       </c>
       <c r="U9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="V9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="W9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>d</v>
       </c>
       <c r="X9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -17262,27 +16296,27 @@
       </c>
       <c r="Y9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>t</v>
       </c>
       <c r="Z9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="AA9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>t</v>
+        <v>q</v>
       </c>
       <c r="AB9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="AC9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="AD9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>d</v>
       </c>
       <c r="AE9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -17290,27 +16324,27 @@
       </c>
       <c r="AF9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>t</v>
       </c>
       <c r="AG9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="AH9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>t</v>
+        <v>q</v>
       </c>
       <c r="AI9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="AJ9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="AK9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>d</v>
       </c>
       <c r="AL9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -17318,27 +16352,27 @@
       </c>
       <c r="AM9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>t</v>
       </c>
       <c r="AN9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="AO9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>t</v>
+        <v>q</v>
       </c>
       <c r="AP9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="AQ9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="AR9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>d</v>
       </c>
       <c r="AS9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -17346,27 +16380,27 @@
       </c>
       <c r="AT9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>t</v>
       </c>
       <c r="AU9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="AV9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>t</v>
+        <v>q</v>
       </c>
       <c r="AW9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="AX9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="AY9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>d</v>
       </c>
       <c r="AZ9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -17374,27 +16408,27 @@
       </c>
       <c r="BA9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>t</v>
       </c>
       <c r="BB9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="BC9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>t</v>
+        <v>q</v>
       </c>
       <c r="BD9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="BE9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="BF9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>d</v>
       </c>
       <c r="BG9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -17402,23 +16436,23 @@
       </c>
       <c r="BH9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>t</v>
       </c>
       <c r="BI9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="BJ9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>t</v>
+        <v>q</v>
       </c>
       <c r="BK9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="BL9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
     </row>
     <row r="10" spans="1:68" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
@@ -17738,7 +16772,7 @@
       </c>
       <c r="F12" s="54">
         <f ca="1">TODAY()</f>
-        <v>46177</v>
+        <v>46179</v>
       </c>
       <c r="G12" s="55">
         <v>3</v>
@@ -17981,7 +17015,7 @@
       <c r="E13" s="53"/>
       <c r="F13" s="54">
         <f ca="1">TODAY()+5</f>
-        <v>46182</v>
+        <v>46184</v>
       </c>
       <c r="G13" s="55">
         <v>1</v>
@@ -18226,7 +17260,7 @@
       </c>
       <c r="F14" s="54">
         <f ca="1">F12-3</f>
-        <v>46174</v>
+        <v>46176</v>
       </c>
       <c r="G14" s="55">
         <v>10</v>
@@ -18469,7 +17503,7 @@
       <c r="E15" s="53"/>
       <c r="F15" s="54">
         <f ca="1">F12+20</f>
-        <v>46197</v>
+        <v>46199</v>
       </c>
       <c r="G15" s="55">
         <v>1</v>
@@ -18714,7 +17748,7 @@
       </c>
       <c r="F16" s="54">
         <f ca="1">F12+6</f>
-        <v>46183</v>
+        <v>46185</v>
       </c>
       <c r="G16" s="55">
         <v>6</v>
@@ -19195,7 +18229,7 @@
       </c>
       <c r="F18" s="54">
         <f ca="1">F12+6</f>
-        <v>46183</v>
+        <v>46185</v>
       </c>
       <c r="G18" s="55">
         <v>13</v>
@@ -19440,7 +18474,7 @@
       </c>
       <c r="F19" s="54">
         <f ca="1">F18+2</f>
-        <v>46185</v>
+        <v>46187</v>
       </c>
       <c r="G19" s="55">
         <v>9</v>
@@ -19685,7 +18719,7 @@
       </c>
       <c r="F20" s="54">
         <f ca="1">F19+5</f>
-        <v>46190</v>
+        <v>46192</v>
       </c>
       <c r="G20" s="55">
         <v>11</v>
@@ -19928,7 +18962,7 @@
       <c r="E21" s="53"/>
       <c r="F21" s="54">
         <f ca="1">F20+2</f>
-        <v>46192</v>
+        <v>46194</v>
       </c>
       <c r="G21" s="55">
         <v>1</v>
@@ -20169,7 +19203,7 @@
       <c r="E22" s="53"/>
       <c r="F22" s="54">
         <f ca="1">F21+1</f>
-        <v>46193</v>
+        <v>46195</v>
       </c>
       <c r="G22" s="55">
         <v>24</v>
@@ -20648,7 +19682,7 @@
       <c r="E24" s="53"/>
       <c r="F24" s="54">
         <f ca="1">F12+15</f>
-        <v>46192</v>
+        <v>46194</v>
       </c>
       <c r="G24" s="55">
         <v>4</v>
@@ -20891,7 +19925,7 @@
       <c r="E25" s="53"/>
       <c r="F25" s="54">
         <f ca="1">F24+3</f>
-        <v>46195</v>
+        <v>46197</v>
       </c>
       <c r="G25" s="55">
         <v>14</v>
@@ -21134,7 +20168,7 @@
       <c r="E26" s="53"/>
       <c r="F26" s="54">
         <f ca="1">F25+15</f>
-        <v>46210</v>
+        <v>46212</v>
       </c>
       <c r="G26" s="55">
         <v>6</v>
@@ -21377,7 +20411,7 @@
       <c r="E27" s="53"/>
       <c r="F27" s="54">
         <f ca="1">F21+22</f>
-        <v>46214</v>
+        <v>46216</v>
       </c>
       <c r="G27" s="55">
         <v>3</v>
@@ -21620,7 +20654,7 @@
       <c r="E28" s="53"/>
       <c r="F28" s="54">
         <f ca="1">F16</f>
-        <v>46183</v>
+        <v>46185</v>
       </c>
       <c r="G28" s="55">
         <v>19</v>
@@ -22097,7 +21131,7 @@
       <c r="E30" s="53"/>
       <c r="F30" s="54">
         <f ca="1">F27+3</f>
-        <v>46217</v>
+        <v>46219</v>
       </c>
       <c r="G30" s="55">
         <v>15</v>
@@ -22338,7 +21372,7 @@
       <c r="E31" s="53"/>
       <c r="F31" s="54">
         <f ca="1">F30+14</f>
-        <v>46231</v>
+        <v>46233</v>
       </c>
       <c r="G31" s="55">
         <v>5</v>
@@ -22581,7 +21615,7 @@
       <c r="E32" s="53"/>
       <c r="F32" s="54">
         <f ca="1">F31+42</f>
-        <v>46273</v>
+        <v>46275</v>
       </c>
       <c r="G32" s="55">
         <v>1</v>
@@ -23621,39 +22655,39 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I6:AM6">
-    <cfRule type="expression" dxfId="89" priority="5">
+    <cfRule type="expression" dxfId="17" priority="5">
       <formula>I$7&lt;=EOMONTH($I$7,0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I6:BL6">
-    <cfRule type="expression" dxfId="88" priority="3">
+    <cfRule type="expression" dxfId="16" priority="3">
       <formula>AND(I$7&lt;=EOMONTH($I$7,1),I$7&gt;EOMONTH($I$7,0))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I7:BL36">
-    <cfRule type="expression" dxfId="87" priority="2">
+    <cfRule type="expression" dxfId="15" priority="2">
       <formula>AND(TODAY()&gt;=I$7,TODAY()&lt;J$7)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I10:BL35">
-    <cfRule type="expression" dxfId="86" priority="8" stopIfTrue="1">
+    <cfRule type="expression" dxfId="14" priority="8" stopIfTrue="1">
       <formula>AND($C10="Baixo risco",I$7&gt;=$F10,I$7&lt;=$F10+$G10-1)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="85" priority="9" stopIfTrue="1">
+    <cfRule type="expression" dxfId="13" priority="9" stopIfTrue="1">
       <formula>AND($C10="Alto risco",I$7&gt;=$F10,I$7&lt;=$F10+$G10-1)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="84" priority="10" stopIfTrue="1">
+    <cfRule type="expression" dxfId="12" priority="10" stopIfTrue="1">
       <formula>AND($C10="No prazo",I$7&gt;=$F10,I$7&lt;=$F10+$G10-1)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="83" priority="11" stopIfTrue="1">
+    <cfRule type="expression" dxfId="11" priority="11" stopIfTrue="1">
       <formula>AND($C10="Médio risco",I$7&gt;=$F10,I$7&lt;=$F10+$G10-1)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="82" priority="12" stopIfTrue="1">
+    <cfRule type="expression" dxfId="10" priority="12" stopIfTrue="1">
       <formula>AND(LEN($C10)=0,I$7&gt;=$F10,I$7&lt;=$F10+$G10-1)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J6:BL6">
-    <cfRule type="expression" dxfId="81" priority="4">
+    <cfRule type="expression" dxfId="9" priority="4">
       <formula>AND(J$7&lt;=EOMONTH($I$7,2),J$7&gt;EOMONTH($I$7,0),J$7&gt;EOMONTH($I$7,1))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -23944,7 +22978,7 @@
       </c>
       <c r="C6" s="71" cm="1">
         <f t="array" aca="1" ref="C6" ca="1">IFERROR(IF(MIN(Milestones43524[Início])=0,TODAY(),B11(Milestones43524[Início])),TODAY())</f>
-        <v>46177</v>
+        <v>46179</v>
       </c>
       <c r="D6" s="72"/>
       <c r="E6" s="66"/>
@@ -24047,227 +23081,227 @@
       <c r="H7" s="74"/>
       <c r="I7" s="106">
         <f ca="1">IFERROR(Início_do_projeto+Incremento_de_Rolagem,TODAY())</f>
-        <v>46178</v>
+        <v>46180</v>
       </c>
       <c r="J7" s="107">
         <f ca="1">I7+1</f>
-        <v>46179</v>
+        <v>46181</v>
       </c>
       <c r="K7" s="107">
         <f t="shared" ref="K7:AX7" ca="1" si="0">J7+1</f>
-        <v>46180</v>
+        <v>46182</v>
       </c>
       <c r="L7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46181</v>
+        <v>46183</v>
       </c>
       <c r="M7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46182</v>
+        <v>46184</v>
       </c>
       <c r="N7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46183</v>
+        <v>46185</v>
       </c>
       <c r="O7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46184</v>
+        <v>46186</v>
       </c>
       <c r="P7" s="107">
         <f ca="1">O7+1</f>
-        <v>46185</v>
+        <v>46187</v>
       </c>
       <c r="Q7" s="107">
         <f ca="1">P7+1</f>
-        <v>46186</v>
+        <v>46188</v>
       </c>
       <c r="R7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46187</v>
+        <v>46189</v>
       </c>
       <c r="S7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46188</v>
+        <v>46190</v>
       </c>
       <c r="T7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46189</v>
+        <v>46191</v>
       </c>
       <c r="U7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46190</v>
+        <v>46192</v>
       </c>
       <c r="V7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46191</v>
+        <v>46193</v>
       </c>
       <c r="W7" s="107">
         <f ca="1">V7+1</f>
-        <v>46192</v>
+        <v>46194</v>
       </c>
       <c r="X7" s="107">
         <f ca="1">W7+1</f>
-        <v>46193</v>
+        <v>46195</v>
       </c>
       <c r="Y7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46194</v>
+        <v>46196</v>
       </c>
       <c r="Z7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46195</v>
+        <v>46197</v>
       </c>
       <c r="AA7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46196</v>
+        <v>46198</v>
       </c>
       <c r="AB7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46197</v>
+        <v>46199</v>
       </c>
       <c r="AC7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46198</v>
+        <v>46200</v>
       </c>
       <c r="AD7" s="107">
         <f ca="1">AC7+1</f>
-        <v>46199</v>
+        <v>46201</v>
       </c>
       <c r="AE7" s="107">
         <f ca="1">AD7+1</f>
-        <v>46200</v>
+        <v>46202</v>
       </c>
       <c r="AF7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46201</v>
+        <v>46203</v>
       </c>
       <c r="AG7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46202</v>
+        <v>46204</v>
       </c>
       <c r="AH7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46203</v>
+        <v>46205</v>
       </c>
       <c r="AI7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46204</v>
+        <v>46206</v>
       </c>
       <c r="AJ7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46205</v>
+        <v>46207</v>
       </c>
       <c r="AK7" s="107">
         <f ca="1">AJ7+1</f>
-        <v>46206</v>
+        <v>46208</v>
       </c>
       <c r="AL7" s="107">
         <f ca="1">AK7+1</f>
-        <v>46207</v>
+        <v>46209</v>
       </c>
       <c r="AM7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46208</v>
+        <v>46210</v>
       </c>
       <c r="AN7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46209</v>
+        <v>46211</v>
       </c>
       <c r="AO7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46210</v>
+        <v>46212</v>
       </c>
       <c r="AP7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46211</v>
+        <v>46213</v>
       </c>
       <c r="AQ7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46212</v>
+        <v>46214</v>
       </c>
       <c r="AR7" s="107">
         <f ca="1">AQ7+1</f>
-        <v>46213</v>
+        <v>46215</v>
       </c>
       <c r="AS7" s="107">
         <f ca="1">AR7+1</f>
-        <v>46214</v>
+        <v>46216</v>
       </c>
       <c r="AT7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46215</v>
+        <v>46217</v>
       </c>
       <c r="AU7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46216</v>
+        <v>46218</v>
       </c>
       <c r="AV7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46217</v>
+        <v>46219</v>
       </c>
       <c r="AW7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46218</v>
+        <v>46220</v>
       </c>
       <c r="AX7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46219</v>
+        <v>46221</v>
       </c>
       <c r="AY7" s="107">
         <f ca="1">AX7+1</f>
-        <v>46220</v>
+        <v>46222</v>
       </c>
       <c r="AZ7" s="107">
         <f ca="1">AY7+1</f>
-        <v>46221</v>
+        <v>46223</v>
       </c>
       <c r="BA7" s="107">
         <f t="shared" ref="BA7:BE7" ca="1" si="1">AZ7+1</f>
-        <v>46222</v>
+        <v>46224</v>
       </c>
       <c r="BB7" s="107">
         <f t="shared" ca="1" si="1"/>
-        <v>46223</v>
+        <v>46225</v>
       </c>
       <c r="BC7" s="107">
         <f t="shared" ca="1" si="1"/>
-        <v>46224</v>
+        <v>46226</v>
       </c>
       <c r="BD7" s="107">
         <f t="shared" ca="1" si="1"/>
-        <v>46225</v>
+        <v>46227</v>
       </c>
       <c r="BE7" s="108">
         <f t="shared" ca="1" si="1"/>
-        <v>46226</v>
+        <v>46228</v>
       </c>
       <c r="BF7" s="107">
         <f ca="1">BE7+1</f>
-        <v>46227</v>
+        <v>46229</v>
       </c>
       <c r="BG7" s="107">
         <f ca="1">BF7+1</f>
-        <v>46228</v>
+        <v>46230</v>
       </c>
       <c r="BH7" s="107">
         <f t="shared" ref="BH7:BL7" ca="1" si="2">BG7+1</f>
-        <v>46229</v>
+        <v>46231</v>
       </c>
       <c r="BI7" s="107">
         <f t="shared" ca="1" si="2"/>
-        <v>46230</v>
+        <v>46232</v>
       </c>
       <c r="BJ7" s="107">
         <f t="shared" ca="1" si="2"/>
-        <v>46231</v>
+        <v>46233</v>
       </c>
       <c r="BK7" s="107">
         <f t="shared" ca="1" si="2"/>
-        <v>46232</v>
+        <v>46234</v>
       </c>
       <c r="BL7" s="108">
         <f t="shared" ca="1" si="2"/>
-        <v>46233</v>
+        <v>46235</v>
       </c>
     </row>
     <row r="8" spans="1:68" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -24359,7 +23393,7 @@
       <c r="H9" s="79"/>
       <c r="I9" s="88" t="str">
         <f t="shared" ref="I9:BL9" ca="1" si="3">LEFT(TEXT(I7,"ddd"),1)</f>
-        <v>s</v>
+        <v>d</v>
       </c>
       <c r="J9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -24367,27 +23401,27 @@
       </c>
       <c r="K9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>t</v>
       </c>
       <c r="L9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="M9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>t</v>
+        <v>q</v>
       </c>
       <c r="N9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="O9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="P9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>d</v>
       </c>
       <c r="Q9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -24395,27 +23429,27 @@
       </c>
       <c r="R9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>t</v>
       </c>
       <c r="S9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="T9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>t</v>
+        <v>q</v>
       </c>
       <c r="U9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="V9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="W9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>d</v>
       </c>
       <c r="X9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -24423,27 +23457,27 @@
       </c>
       <c r="Y9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>t</v>
       </c>
       <c r="Z9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="AA9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>t</v>
+        <v>q</v>
       </c>
       <c r="AB9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="AC9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="AD9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>d</v>
       </c>
       <c r="AE9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -24451,27 +23485,27 @@
       </c>
       <c r="AF9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>t</v>
       </c>
       <c r="AG9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="AH9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>t</v>
+        <v>q</v>
       </c>
       <c r="AI9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="AJ9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="AK9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>d</v>
       </c>
       <c r="AL9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -24479,27 +23513,27 @@
       </c>
       <c r="AM9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>t</v>
       </c>
       <c r="AN9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="AO9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>t</v>
+        <v>q</v>
       </c>
       <c r="AP9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="AQ9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="AR9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>d</v>
       </c>
       <c r="AS9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -24507,27 +23541,27 @@
       </c>
       <c r="AT9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>t</v>
       </c>
       <c r="AU9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="AV9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>t</v>
+        <v>q</v>
       </c>
       <c r="AW9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="AX9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="AY9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>d</v>
       </c>
       <c r="AZ9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -24535,27 +23569,27 @@
       </c>
       <c r="BA9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>t</v>
       </c>
       <c r="BB9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="BC9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>t</v>
+        <v>q</v>
       </c>
       <c r="BD9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="BE9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="BF9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>d</v>
       </c>
       <c r="BG9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -24563,23 +23597,23 @@
       </c>
       <c r="BH9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>t</v>
       </c>
       <c r="BI9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="BJ9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>t</v>
+        <v>q</v>
       </c>
       <c r="BK9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="BL9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
     </row>
     <row r="10" spans="1:68" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
@@ -24899,7 +23933,7 @@
       </c>
       <c r="F12" s="54">
         <f ca="1">TODAY()</f>
-        <v>46177</v>
+        <v>46179</v>
       </c>
       <c r="G12" s="55">
         <v>3</v>
@@ -25142,7 +24176,7 @@
       <c r="E13" s="53"/>
       <c r="F13" s="54">
         <f ca="1">TODAY()+5</f>
-        <v>46182</v>
+        <v>46184</v>
       </c>
       <c r="G13" s="55">
         <v>1</v>
@@ -25387,7 +24421,7 @@
       </c>
       <c r="F14" s="54">
         <f ca="1">F12-3</f>
-        <v>46174</v>
+        <v>46176</v>
       </c>
       <c r="G14" s="55">
         <v>10</v>
@@ -25630,7 +24664,7 @@
       <c r="E15" s="53"/>
       <c r="F15" s="54">
         <f ca="1">F12+20</f>
-        <v>46197</v>
+        <v>46199</v>
       </c>
       <c r="G15" s="55">
         <v>1</v>
@@ -25875,7 +24909,7 @@
       </c>
       <c r="F16" s="54">
         <f ca="1">F12+6</f>
-        <v>46183</v>
+        <v>46185</v>
       </c>
       <c r="G16" s="55">
         <v>6</v>
@@ -26356,7 +25390,7 @@
       </c>
       <c r="F18" s="54">
         <f ca="1">F12+6</f>
-        <v>46183</v>
+        <v>46185</v>
       </c>
       <c r="G18" s="55">
         <v>13</v>
@@ -26601,7 +25635,7 @@
       </c>
       <c r="F19" s="54">
         <f ca="1">F18+2</f>
-        <v>46185</v>
+        <v>46187</v>
       </c>
       <c r="G19" s="55">
         <v>9</v>
@@ -26846,7 +25880,7 @@
       </c>
       <c r="F20" s="54">
         <f ca="1">F19+5</f>
-        <v>46190</v>
+        <v>46192</v>
       </c>
       <c r="G20" s="55">
         <v>11</v>
@@ -27089,7 +26123,7 @@
       <c r="E21" s="53"/>
       <c r="F21" s="54">
         <f ca="1">F20+2</f>
-        <v>46192</v>
+        <v>46194</v>
       </c>
       <c r="G21" s="55">
         <v>1</v>
@@ -27330,7 +26364,7 @@
       <c r="E22" s="53"/>
       <c r="F22" s="54">
         <f ca="1">F21+1</f>
-        <v>46193</v>
+        <v>46195</v>
       </c>
       <c r="G22" s="55">
         <v>24</v>
@@ -27809,7 +26843,7 @@
       <c r="E24" s="53"/>
       <c r="F24" s="54">
         <f ca="1">F12+15</f>
-        <v>46192</v>
+        <v>46194</v>
       </c>
       <c r="G24" s="55">
         <v>4</v>
@@ -28052,7 +27086,7 @@
       <c r="E25" s="53"/>
       <c r="F25" s="54">
         <f ca="1">F24+3</f>
-        <v>46195</v>
+        <v>46197</v>
       </c>
       <c r="G25" s="55">
         <v>14</v>
@@ -28295,7 +27329,7 @@
       <c r="E26" s="53"/>
       <c r="F26" s="54">
         <f ca="1">F25+15</f>
-        <v>46210</v>
+        <v>46212</v>
       </c>
       <c r="G26" s="55">
         <v>6</v>
@@ -28538,7 +27572,7 @@
       <c r="E27" s="53"/>
       <c r="F27" s="54">
         <f ca="1">F21+22</f>
-        <v>46214</v>
+        <v>46216</v>
       </c>
       <c r="G27" s="55">
         <v>3</v>
@@ -28781,7 +27815,7 @@
       <c r="E28" s="53"/>
       <c r="F28" s="54">
         <f ca="1">F16</f>
-        <v>46183</v>
+        <v>46185</v>
       </c>
       <c r="G28" s="55">
         <v>19</v>
@@ -29258,7 +28292,7 @@
       <c r="E30" s="53"/>
       <c r="F30" s="54">
         <f ca="1">F27+3</f>
-        <v>46217</v>
+        <v>46219</v>
       </c>
       <c r="G30" s="55">
         <v>15</v>
@@ -29499,7 +28533,7 @@
       <c r="E31" s="53"/>
       <c r="F31" s="54">
         <f ca="1">F30+14</f>
-        <v>46231</v>
+        <v>46233</v>
       </c>
       <c r="G31" s="55">
         <v>5</v>
@@ -29742,7 +28776,7 @@
       <c r="E32" s="53"/>
       <c r="F32" s="54">
         <f ca="1">F31+42</f>
-        <v>46273</v>
+        <v>46275</v>
       </c>
       <c r="G32" s="55">
         <v>1</v>
@@ -30782,39 +29816,39 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I6:AM6">
-    <cfRule type="expression" dxfId="80" priority="4">
+    <cfRule type="expression" dxfId="8" priority="4">
       <formula>I$7&lt;=EOMONTH($I$7,0)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I6:BL6">
-    <cfRule type="expression" dxfId="79" priority="2">
+    <cfRule type="expression" dxfId="7" priority="2">
       <formula>AND(I$7&lt;=EOMONTH($I$7,1),I$7&gt;EOMONTH($I$7,0))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I7:BL36">
-    <cfRule type="expression" dxfId="78" priority="1">
+    <cfRule type="expression" dxfId="6" priority="1">
       <formula>AND(TODAY()&gt;=I$7,TODAY()&lt;J$7)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I10:BL35">
-    <cfRule type="expression" dxfId="77" priority="7" stopIfTrue="1">
+    <cfRule type="expression" dxfId="5" priority="7" stopIfTrue="1">
       <formula>AND($C10="Baixo risco",I$7&gt;=$F10,I$7&lt;=$F10+$G10-1)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="76" priority="8" stopIfTrue="1">
+    <cfRule type="expression" dxfId="4" priority="8" stopIfTrue="1">
       <formula>AND($C10="Alto risco",I$7&gt;=$F10,I$7&lt;=$F10+$G10-1)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="75" priority="9" stopIfTrue="1">
+    <cfRule type="expression" dxfId="3" priority="9" stopIfTrue="1">
       <formula>AND($C10="No prazo",I$7&gt;=$F10,I$7&lt;=$F10+$G10-1)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="74" priority="10" stopIfTrue="1">
+    <cfRule type="expression" dxfId="2" priority="10" stopIfTrue="1">
       <formula>AND($C10="Médio risco",I$7&gt;=$F10,I$7&lt;=$F10+$G10-1)</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="73" priority="11" stopIfTrue="1">
+    <cfRule type="expression" dxfId="1" priority="11" stopIfTrue="1">
       <formula>AND(LEN($C10)=0,I$7&gt;=$F10,I$7&lt;=$F10+$G10-1)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J6:BL6">
-    <cfRule type="expression" dxfId="72" priority="3">
+    <cfRule type="expression" dxfId="0" priority="3">
       <formula>AND(J$7&lt;=EOMONTH($I$7,2),J$7&gt;EOMONTH($I$7,0),J$7&gt;EOMONTH($I$7,1))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -30937,6 +29971,34 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Url xsi:nil="true"/>
+      <Description xsi:nil="true"/>
+    </Image>
+    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
+    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010079F111ED35F8CC479449609E8A0923A6" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="22a266b9fa9a230c5a512669d8b298c3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xmlns:ns3="16c05727-aa75-4e4a-9b5f-8a80a1165891" xmlns:ns4="230e9df3-be65-4c73-a93b-d1236ebd677e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="eddc33fff6b14141ee5c74a0d29ea6a1" ns1:_="" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -31212,35 +30274,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA4BA2A8-DB97-40F9-8DB6-154C09C7467C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
+    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Url xsi:nil="true"/>
-      <Description xsi:nil="true"/>
-    </Image>
-    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
-    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{39060724-9CA2-4290-8A0C-B53624A594E7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{75C87518-DD8E-42CD-8DAC-291A323E849B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -31259,24 +30313,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{39060724-9CA2-4290-8A0C-B53624A594E7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA4BA2A8-DB97-40F9-8DB6-154C09C7467C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
-    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Add SD-005 Design Telemetry Aggregation Service
</commit_message>
<xml_diff>
--- a/docs/0004-gant-doc.xlsx
+++ b/docs/0004-gant-doc.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{397539F9-548B-4B68-A831-E42ECC6A5A7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8B5D120-481B-416B-88A3-DC166C7A69DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="415" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6570,7 +6570,7 @@
         <v>38</v>
       </c>
       <c r="D16" s="19" t="s">
-        <v>23</v>
+        <v>122</v>
       </c>
       <c r="E16" s="19" t="s">
         <v>53</v>
@@ -6598,9 +6598,9 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-      <c r="M16" s="40" t="str">
-        <f t="shared" ca="1" si="4"/>
-        <v/>
+      <c r="M16" s="40">
+        <f t="shared" ca="1" si="4"/>
+        <v>0</v>
       </c>
       <c r="N16" s="40" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -6610,9 +6610,9 @@
         <f t="shared" ca="1" si="4"/>
         <v/>
       </c>
-      <c r="P16" s="40" t="str">
-        <f t="shared" ca="1" si="4"/>
-        <v/>
+      <c r="P16" s="40">
+        <f t="shared" ca="1" si="4"/>
+        <v>0</v>
       </c>
       <c r="Q16" s="40" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -16087,7 +16087,7 @@
       </c>
       <c r="C6" s="71" cm="1">
         <f t="array" aca="1" ref="C6" ca="1">IFERROR(IF(MIN(Milestones4352[Início])=0,TODAY(),B11(Milestones4352[Início])),TODAY())</f>
-        <v>46189</v>
+        <v>46201</v>
       </c>
       <c r="D6" s="72"/>
       <c r="E6" s="66"/>
@@ -16106,7 +16106,7 @@
       <c r="O6" s="82"/>
       <c r="P6" s="82" t="str">
         <f ca="1">IF(TEXT(P7,"mmmm")=I6,"",TEXT(P7,"mmmm"))</f>
-        <v/>
+        <v>julho</v>
       </c>
       <c r="Q6" s="82"/>
       <c r="R6" s="82"/>
@@ -16116,7 +16116,7 @@
       <c r="V6" s="82"/>
       <c r="W6" s="82" t="str">
         <f ca="1">IF(OR(TEXT(W7,"mmmm")=P6,TEXT(W7,"mmmm")=I6),"",TEXT(W7,"mmmm"))</f>
-        <v>julho</v>
+        <v/>
       </c>
       <c r="X6" s="82"/>
       <c r="Y6" s="82"/>
@@ -16146,7 +16146,7 @@
       <c r="AQ6" s="82"/>
       <c r="AR6" s="82" t="str">
         <f ca="1">IF(OR(TEXT(AR7,"mmmm")=AK6,TEXT(AR7,"mmmm")=AD6,TEXT(AR7,"mmmm")=W6,TEXT(AR7,"mmmm")=P6),"",TEXT(AR7,"mmmm"))</f>
-        <v/>
+        <v>agosto</v>
       </c>
       <c r="AS6" s="82"/>
       <c r="AT6" s="82"/>
@@ -16166,7 +16166,7 @@
       <c r="BE6" s="81"/>
       <c r="BF6" s="81" t="str">
         <f ca="1">IF(OR(TEXT(BF7,"mmmm")=AY6,TEXT(BF7,"mmmm")=AR6,TEXT(BF7,"mmmm")=AK6,TEXT(BF7,"mmmm")=AD6),"",TEXT(BF7,"mmmm"))</f>
-        <v>agosto</v>
+        <v/>
       </c>
       <c r="BG6" s="81"/>
       <c r="BH6" s="81"/>
@@ -16190,227 +16190,227 @@
       <c r="H7" s="74"/>
       <c r="I7" s="106">
         <f ca="1">IFERROR(Início_do_projeto+Incremento_de_Rolagem,TODAY())</f>
-        <v>46190</v>
+        <v>46202</v>
       </c>
       <c r="J7" s="107">
         <f ca="1">I7+1</f>
-        <v>46191</v>
+        <v>46203</v>
       </c>
       <c r="K7" s="107">
         <f t="shared" ref="K7:AX7" ca="1" si="0">J7+1</f>
-        <v>46192</v>
+        <v>46204</v>
       </c>
       <c r="L7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46193</v>
+        <v>46205</v>
       </c>
       <c r="M7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46194</v>
+        <v>46206</v>
       </c>
       <c r="N7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46195</v>
+        <v>46207</v>
       </c>
       <c r="O7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46196</v>
+        <v>46208</v>
       </c>
       <c r="P7" s="107">
         <f ca="1">O7+1</f>
-        <v>46197</v>
+        <v>46209</v>
       </c>
       <c r="Q7" s="107">
         <f ca="1">P7+1</f>
-        <v>46198</v>
+        <v>46210</v>
       </c>
       <c r="R7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46199</v>
+        <v>46211</v>
       </c>
       <c r="S7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46200</v>
+        <v>46212</v>
       </c>
       <c r="T7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46201</v>
+        <v>46213</v>
       </c>
       <c r="U7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46202</v>
+        <v>46214</v>
       </c>
       <c r="V7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46203</v>
+        <v>46215</v>
       </c>
       <c r="W7" s="107">
         <f ca="1">V7+1</f>
-        <v>46204</v>
+        <v>46216</v>
       </c>
       <c r="X7" s="107">
         <f ca="1">W7+1</f>
-        <v>46205</v>
+        <v>46217</v>
       </c>
       <c r="Y7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46206</v>
+        <v>46218</v>
       </c>
       <c r="Z7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46207</v>
+        <v>46219</v>
       </c>
       <c r="AA7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46208</v>
+        <v>46220</v>
       </c>
       <c r="AB7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46209</v>
+        <v>46221</v>
       </c>
       <c r="AC7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46210</v>
+        <v>46222</v>
       </c>
       <c r="AD7" s="107">
         <f ca="1">AC7+1</f>
-        <v>46211</v>
+        <v>46223</v>
       </c>
       <c r="AE7" s="107">
         <f ca="1">AD7+1</f>
-        <v>46212</v>
+        <v>46224</v>
       </c>
       <c r="AF7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46213</v>
+        <v>46225</v>
       </c>
       <c r="AG7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46214</v>
+        <v>46226</v>
       </c>
       <c r="AH7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46215</v>
+        <v>46227</v>
       </c>
       <c r="AI7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46216</v>
+        <v>46228</v>
       </c>
       <c r="AJ7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46217</v>
+        <v>46229</v>
       </c>
       <c r="AK7" s="107">
         <f ca="1">AJ7+1</f>
-        <v>46218</v>
+        <v>46230</v>
       </c>
       <c r="AL7" s="107">
         <f ca="1">AK7+1</f>
-        <v>46219</v>
+        <v>46231</v>
       </c>
       <c r="AM7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46220</v>
+        <v>46232</v>
       </c>
       <c r="AN7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46221</v>
+        <v>46233</v>
       </c>
       <c r="AO7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46222</v>
+        <v>46234</v>
       </c>
       <c r="AP7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46223</v>
+        <v>46235</v>
       </c>
       <c r="AQ7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46224</v>
+        <v>46236</v>
       </c>
       <c r="AR7" s="107">
         <f ca="1">AQ7+1</f>
-        <v>46225</v>
+        <v>46237</v>
       </c>
       <c r="AS7" s="107">
         <f ca="1">AR7+1</f>
-        <v>46226</v>
+        <v>46238</v>
       </c>
       <c r="AT7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46227</v>
+        <v>46239</v>
       </c>
       <c r="AU7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46228</v>
+        <v>46240</v>
       </c>
       <c r="AV7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46229</v>
+        <v>46241</v>
       </c>
       <c r="AW7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46230</v>
+        <v>46242</v>
       </c>
       <c r="AX7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46231</v>
+        <v>46243</v>
       </c>
       <c r="AY7" s="107">
         <f ca="1">AX7+1</f>
-        <v>46232</v>
+        <v>46244</v>
       </c>
       <c r="AZ7" s="107">
         <f ca="1">AY7+1</f>
-        <v>46233</v>
+        <v>46245</v>
       </c>
       <c r="BA7" s="107">
         <f t="shared" ref="BA7:BE7" ca="1" si="1">AZ7+1</f>
-        <v>46234</v>
+        <v>46246</v>
       </c>
       <c r="BB7" s="107">
         <f t="shared" ca="1" si="1"/>
-        <v>46235</v>
+        <v>46247</v>
       </c>
       <c r="BC7" s="107">
         <f t="shared" ca="1" si="1"/>
-        <v>46236</v>
+        <v>46248</v>
       </c>
       <c r="BD7" s="107">
         <f t="shared" ca="1" si="1"/>
-        <v>46237</v>
+        <v>46249</v>
       </c>
       <c r="BE7" s="108">
         <f t="shared" ca="1" si="1"/>
-        <v>46238</v>
+        <v>46250</v>
       </c>
       <c r="BF7" s="107">
         <f ca="1">BE7+1</f>
-        <v>46239</v>
+        <v>46251</v>
       </c>
       <c r="BG7" s="107">
         <f ca="1">BF7+1</f>
-        <v>46240</v>
+        <v>46252</v>
       </c>
       <c r="BH7" s="107">
         <f t="shared" ref="BH7:BL7" ca="1" si="2">BG7+1</f>
-        <v>46241</v>
+        <v>46253</v>
       </c>
       <c r="BI7" s="107">
         <f t="shared" ca="1" si="2"/>
-        <v>46242</v>
+        <v>46254</v>
       </c>
       <c r="BJ7" s="107">
         <f t="shared" ca="1" si="2"/>
-        <v>46243</v>
+        <v>46255</v>
       </c>
       <c r="BK7" s="107">
         <f t="shared" ca="1" si="2"/>
-        <v>46244</v>
+        <v>46256</v>
       </c>
       <c r="BL7" s="108">
         <f t="shared" ca="1" si="2"/>
-        <v>46245</v>
+        <v>46257</v>
       </c>
     </row>
     <row r="8" spans="1:68" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -16502,23 +16502,23 @@
       <c r="H9" s="79"/>
       <c r="I9" s="88" t="str">
         <f t="shared" ref="I9:BL9" ca="1" si="3">LEFT(TEXT(I7,"ddd"),1)</f>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="J9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>t</v>
       </c>
       <c r="K9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="L9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="M9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>s</v>
       </c>
       <c r="N9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -16526,27 +16526,27 @@
       </c>
       <c r="O9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>t</v>
+        <v>d</v>
       </c>
       <c r="P9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="Q9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>t</v>
       </c>
       <c r="R9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="S9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="T9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>s</v>
       </c>
       <c r="U9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -16554,27 +16554,27 @@
       </c>
       <c r="V9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>t</v>
+        <v>d</v>
       </c>
       <c r="W9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="X9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>t</v>
       </c>
       <c r="Y9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="Z9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="AA9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>s</v>
       </c>
       <c r="AB9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -16582,27 +16582,27 @@
       </c>
       <c r="AC9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>t</v>
+        <v>d</v>
       </c>
       <c r="AD9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="AE9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>t</v>
       </c>
       <c r="AF9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="AG9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="AH9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>s</v>
       </c>
       <c r="AI9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -16610,27 +16610,27 @@
       </c>
       <c r="AJ9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>t</v>
+        <v>d</v>
       </c>
       <c r="AK9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="AL9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>t</v>
       </c>
       <c r="AM9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="AN9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="AO9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>s</v>
       </c>
       <c r="AP9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -16638,27 +16638,27 @@
       </c>
       <c r="AQ9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>t</v>
+        <v>d</v>
       </c>
       <c r="AR9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="AS9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>t</v>
       </c>
       <c r="AT9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="AU9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="AV9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>s</v>
       </c>
       <c r="AW9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -16666,27 +16666,27 @@
       </c>
       <c r="AX9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>t</v>
+        <v>d</v>
       </c>
       <c r="AY9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="AZ9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>t</v>
       </c>
       <c r="BA9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="BB9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="BC9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>s</v>
       </c>
       <c r="BD9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -16694,27 +16694,27 @@
       </c>
       <c r="BE9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>t</v>
+        <v>d</v>
       </c>
       <c r="BF9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="BG9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>t</v>
       </c>
       <c r="BH9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="BI9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="BJ9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>s</v>
       </c>
       <c r="BK9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -16722,7 +16722,7 @@
       </c>
       <c r="BL9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>t</v>
+        <v>d</v>
       </c>
     </row>
     <row r="10" spans="1:68" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
@@ -17042,7 +17042,7 @@
       </c>
       <c r="F12" s="54">
         <f ca="1">TODAY()</f>
-        <v>46189</v>
+        <v>46201</v>
       </c>
       <c r="G12" s="55">
         <v>3</v>
@@ -17285,7 +17285,7 @@
       <c r="E13" s="53"/>
       <c r="F13" s="54">
         <f ca="1">TODAY()+5</f>
-        <v>46194</v>
+        <v>46206</v>
       </c>
       <c r="G13" s="55">
         <v>1</v>
@@ -17530,7 +17530,7 @@
       </c>
       <c r="F14" s="54">
         <f ca="1">F12-3</f>
-        <v>46186</v>
+        <v>46198</v>
       </c>
       <c r="G14" s="55">
         <v>10</v>
@@ -17773,7 +17773,7 @@
       <c r="E15" s="53"/>
       <c r="F15" s="54">
         <f ca="1">F12+20</f>
-        <v>46209</v>
+        <v>46221</v>
       </c>
       <c r="G15" s="55">
         <v>1</v>
@@ -18018,7 +18018,7 @@
       </c>
       <c r="F16" s="54">
         <f ca="1">F12+6</f>
-        <v>46195</v>
+        <v>46207</v>
       </c>
       <c r="G16" s="55">
         <v>6</v>
@@ -18499,7 +18499,7 @@
       </c>
       <c r="F18" s="54">
         <f ca="1">F12+6</f>
-        <v>46195</v>
+        <v>46207</v>
       </c>
       <c r="G18" s="55">
         <v>13</v>
@@ -18744,7 +18744,7 @@
       </c>
       <c r="F19" s="54">
         <f ca="1">F18+2</f>
-        <v>46197</v>
+        <v>46209</v>
       </c>
       <c r="G19" s="55">
         <v>9</v>
@@ -18989,7 +18989,7 @@
       </c>
       <c r="F20" s="54">
         <f ca="1">F19+5</f>
-        <v>46202</v>
+        <v>46214</v>
       </c>
       <c r="G20" s="55">
         <v>11</v>
@@ -19232,7 +19232,7 @@
       <c r="E21" s="53"/>
       <c r="F21" s="54">
         <f ca="1">F20+2</f>
-        <v>46204</v>
+        <v>46216</v>
       </c>
       <c r="G21" s="55">
         <v>1</v>
@@ -19473,7 +19473,7 @@
       <c r="E22" s="53"/>
       <c r="F22" s="54">
         <f ca="1">F21+1</f>
-        <v>46205</v>
+        <v>46217</v>
       </c>
       <c r="G22" s="55">
         <v>24</v>
@@ -19952,7 +19952,7 @@
       <c r="E24" s="53"/>
       <c r="F24" s="54">
         <f ca="1">F12+15</f>
-        <v>46204</v>
+        <v>46216</v>
       </c>
       <c r="G24" s="55">
         <v>4</v>
@@ -20195,7 +20195,7 @@
       <c r="E25" s="53"/>
       <c r="F25" s="54">
         <f ca="1">F24+3</f>
-        <v>46207</v>
+        <v>46219</v>
       </c>
       <c r="G25" s="55">
         <v>14</v>
@@ -20438,7 +20438,7 @@
       <c r="E26" s="53"/>
       <c r="F26" s="54">
         <f ca="1">F25+15</f>
-        <v>46222</v>
+        <v>46234</v>
       </c>
       <c r="G26" s="55">
         <v>6</v>
@@ -20681,7 +20681,7 @@
       <c r="E27" s="53"/>
       <c r="F27" s="54">
         <f ca="1">F21+22</f>
-        <v>46226</v>
+        <v>46238</v>
       </c>
       <c r="G27" s="55">
         <v>3</v>
@@ -20924,7 +20924,7 @@
       <c r="E28" s="53"/>
       <c r="F28" s="54">
         <f ca="1">F16</f>
-        <v>46195</v>
+        <v>46207</v>
       </c>
       <c r="G28" s="55">
         <v>19</v>
@@ -21401,7 +21401,7 @@
       <c r="E30" s="53"/>
       <c r="F30" s="54">
         <f ca="1">F27+3</f>
-        <v>46229</v>
+        <v>46241</v>
       </c>
       <c r="G30" s="55">
         <v>15</v>
@@ -21642,7 +21642,7 @@
       <c r="E31" s="53"/>
       <c r="F31" s="54">
         <f ca="1">F30+14</f>
-        <v>46243</v>
+        <v>46255</v>
       </c>
       <c r="G31" s="55">
         <v>5</v>
@@ -21885,7 +21885,7 @@
       <c r="E32" s="53"/>
       <c r="F32" s="54">
         <f ca="1">F31+42</f>
-        <v>46285</v>
+        <v>46297</v>
       </c>
       <c r="G32" s="55">
         <v>1</v>
@@ -23248,7 +23248,7 @@
       </c>
       <c r="C6" s="71" cm="1">
         <f t="array" aca="1" ref="C6" ca="1">IFERROR(IF(MIN(Milestones43524[Início])=0,TODAY(),B11(Milestones43524[Início])),TODAY())</f>
-        <v>46189</v>
+        <v>46201</v>
       </c>
       <c r="D6" s="72"/>
       <c r="E6" s="66"/>
@@ -23267,7 +23267,7 @@
       <c r="O6" s="82"/>
       <c r="P6" s="82" t="str">
         <f ca="1">IF(TEXT(P7,"mmmm")=I6,"",TEXT(P7,"mmmm"))</f>
-        <v/>
+        <v>julho</v>
       </c>
       <c r="Q6" s="82"/>
       <c r="R6" s="82"/>
@@ -23277,7 +23277,7 @@
       <c r="V6" s="82"/>
       <c r="W6" s="82" t="str">
         <f ca="1">IF(OR(TEXT(W7,"mmmm")=P6,TEXT(W7,"mmmm")=I6),"",TEXT(W7,"mmmm"))</f>
-        <v>julho</v>
+        <v/>
       </c>
       <c r="X6" s="82"/>
       <c r="Y6" s="82"/>
@@ -23307,7 +23307,7 @@
       <c r="AQ6" s="82"/>
       <c r="AR6" s="82" t="str">
         <f ca="1">IF(OR(TEXT(AR7,"mmmm")=AK6,TEXT(AR7,"mmmm")=AD6,TEXT(AR7,"mmmm")=W6,TEXT(AR7,"mmmm")=P6),"",TEXT(AR7,"mmmm"))</f>
-        <v/>
+        <v>agosto</v>
       </c>
       <c r="AS6" s="82"/>
       <c r="AT6" s="82"/>
@@ -23327,7 +23327,7 @@
       <c r="BE6" s="81"/>
       <c r="BF6" s="81" t="str">
         <f ca="1">IF(OR(TEXT(BF7,"mmmm")=AY6,TEXT(BF7,"mmmm")=AR6,TEXT(BF7,"mmmm")=AK6,TEXT(BF7,"mmmm")=AD6),"",TEXT(BF7,"mmmm"))</f>
-        <v>agosto</v>
+        <v/>
       </c>
       <c r="BG6" s="81"/>
       <c r="BH6" s="81"/>
@@ -23351,227 +23351,227 @@
       <c r="H7" s="74"/>
       <c r="I7" s="106">
         <f ca="1">IFERROR(Início_do_projeto+Incremento_de_Rolagem,TODAY())</f>
-        <v>46190</v>
+        <v>46202</v>
       </c>
       <c r="J7" s="107">
         <f ca="1">I7+1</f>
-        <v>46191</v>
+        <v>46203</v>
       </c>
       <c r="K7" s="107">
         <f t="shared" ref="K7:AX7" ca="1" si="0">J7+1</f>
-        <v>46192</v>
+        <v>46204</v>
       </c>
       <c r="L7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46193</v>
+        <v>46205</v>
       </c>
       <c r="M7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46194</v>
+        <v>46206</v>
       </c>
       <c r="N7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46195</v>
+        <v>46207</v>
       </c>
       <c r="O7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46196</v>
+        <v>46208</v>
       </c>
       <c r="P7" s="107">
         <f ca="1">O7+1</f>
-        <v>46197</v>
+        <v>46209</v>
       </c>
       <c r="Q7" s="107">
         <f ca="1">P7+1</f>
-        <v>46198</v>
+        <v>46210</v>
       </c>
       <c r="R7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46199</v>
+        <v>46211</v>
       </c>
       <c r="S7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46200</v>
+        <v>46212</v>
       </c>
       <c r="T7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46201</v>
+        <v>46213</v>
       </c>
       <c r="U7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46202</v>
+        <v>46214</v>
       </c>
       <c r="V7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46203</v>
+        <v>46215</v>
       </c>
       <c r="W7" s="107">
         <f ca="1">V7+1</f>
-        <v>46204</v>
+        <v>46216</v>
       </c>
       <c r="X7" s="107">
         <f ca="1">W7+1</f>
-        <v>46205</v>
+        <v>46217</v>
       </c>
       <c r="Y7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46206</v>
+        <v>46218</v>
       </c>
       <c r="Z7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46207</v>
+        <v>46219</v>
       </c>
       <c r="AA7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46208</v>
+        <v>46220</v>
       </c>
       <c r="AB7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46209</v>
+        <v>46221</v>
       </c>
       <c r="AC7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46210</v>
+        <v>46222</v>
       </c>
       <c r="AD7" s="107">
         <f ca="1">AC7+1</f>
-        <v>46211</v>
+        <v>46223</v>
       </c>
       <c r="AE7" s="107">
         <f ca="1">AD7+1</f>
-        <v>46212</v>
+        <v>46224</v>
       </c>
       <c r="AF7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46213</v>
+        <v>46225</v>
       </c>
       <c r="AG7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46214</v>
+        <v>46226</v>
       </c>
       <c r="AH7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46215</v>
+        <v>46227</v>
       </c>
       <c r="AI7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46216</v>
+        <v>46228</v>
       </c>
       <c r="AJ7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46217</v>
+        <v>46229</v>
       </c>
       <c r="AK7" s="107">
         <f ca="1">AJ7+1</f>
-        <v>46218</v>
+        <v>46230</v>
       </c>
       <c r="AL7" s="107">
         <f ca="1">AK7+1</f>
-        <v>46219</v>
+        <v>46231</v>
       </c>
       <c r="AM7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46220</v>
+        <v>46232</v>
       </c>
       <c r="AN7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46221</v>
+        <v>46233</v>
       </c>
       <c r="AO7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46222</v>
+        <v>46234</v>
       </c>
       <c r="AP7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46223</v>
+        <v>46235</v>
       </c>
       <c r="AQ7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46224</v>
+        <v>46236</v>
       </c>
       <c r="AR7" s="107">
         <f ca="1">AQ7+1</f>
-        <v>46225</v>
+        <v>46237</v>
       </c>
       <c r="AS7" s="107">
         <f ca="1">AR7+1</f>
-        <v>46226</v>
+        <v>46238</v>
       </c>
       <c r="AT7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46227</v>
+        <v>46239</v>
       </c>
       <c r="AU7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46228</v>
+        <v>46240</v>
       </c>
       <c r="AV7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46229</v>
+        <v>46241</v>
       </c>
       <c r="AW7" s="107">
         <f t="shared" ca="1" si="0"/>
-        <v>46230</v>
+        <v>46242</v>
       </c>
       <c r="AX7" s="108">
         <f t="shared" ca="1" si="0"/>
-        <v>46231</v>
+        <v>46243</v>
       </c>
       <c r="AY7" s="107">
         <f ca="1">AX7+1</f>
-        <v>46232</v>
+        <v>46244</v>
       </c>
       <c r="AZ7" s="107">
         <f ca="1">AY7+1</f>
-        <v>46233</v>
+        <v>46245</v>
       </c>
       <c r="BA7" s="107">
         <f t="shared" ref="BA7:BE7" ca="1" si="1">AZ7+1</f>
-        <v>46234</v>
+        <v>46246</v>
       </c>
       <c r="BB7" s="107">
         <f t="shared" ca="1" si="1"/>
-        <v>46235</v>
+        <v>46247</v>
       </c>
       <c r="BC7" s="107">
         <f t="shared" ca="1" si="1"/>
-        <v>46236</v>
+        <v>46248</v>
       </c>
       <c r="BD7" s="107">
         <f t="shared" ca="1" si="1"/>
-        <v>46237</v>
+        <v>46249</v>
       </c>
       <c r="BE7" s="108">
         <f t="shared" ca="1" si="1"/>
-        <v>46238</v>
+        <v>46250</v>
       </c>
       <c r="BF7" s="107">
         <f ca="1">BE7+1</f>
-        <v>46239</v>
+        <v>46251</v>
       </c>
       <c r="BG7" s="107">
         <f ca="1">BF7+1</f>
-        <v>46240</v>
+        <v>46252</v>
       </c>
       <c r="BH7" s="107">
         <f t="shared" ref="BH7:BL7" ca="1" si="2">BG7+1</f>
-        <v>46241</v>
+        <v>46253</v>
       </c>
       <c r="BI7" s="107">
         <f t="shared" ca="1" si="2"/>
-        <v>46242</v>
+        <v>46254</v>
       </c>
       <c r="BJ7" s="107">
         <f t="shared" ca="1" si="2"/>
-        <v>46243</v>
+        <v>46255</v>
       </c>
       <c r="BK7" s="107">
         <f t="shared" ca="1" si="2"/>
-        <v>46244</v>
+        <v>46256</v>
       </c>
       <c r="BL7" s="108">
         <f t="shared" ca="1" si="2"/>
-        <v>46245</v>
+        <v>46257</v>
       </c>
     </row>
     <row r="8" spans="1:68" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -23663,23 +23663,23 @@
       <c r="H9" s="79"/>
       <c r="I9" s="88" t="str">
         <f t="shared" ref="I9:BL9" ca="1" si="3">LEFT(TEXT(I7,"ddd"),1)</f>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="J9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>t</v>
       </c>
       <c r="K9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="L9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="M9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>s</v>
       </c>
       <c r="N9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -23687,27 +23687,27 @@
       </c>
       <c r="O9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>t</v>
+        <v>d</v>
       </c>
       <c r="P9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="Q9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>t</v>
       </c>
       <c r="R9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="S9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="T9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>s</v>
       </c>
       <c r="U9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -23715,27 +23715,27 @@
       </c>
       <c r="V9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>t</v>
+        <v>d</v>
       </c>
       <c r="W9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="X9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>t</v>
       </c>
       <c r="Y9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="Z9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="AA9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>s</v>
       </c>
       <c r="AB9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -23743,27 +23743,27 @@
       </c>
       <c r="AC9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>t</v>
+        <v>d</v>
       </c>
       <c r="AD9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="AE9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>t</v>
       </c>
       <c r="AF9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="AG9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="AH9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>s</v>
       </c>
       <c r="AI9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -23771,27 +23771,27 @@
       </c>
       <c r="AJ9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>t</v>
+        <v>d</v>
       </c>
       <c r="AK9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="AL9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>t</v>
       </c>
       <c r="AM9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="AN9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="AO9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>s</v>
       </c>
       <c r="AP9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -23799,27 +23799,27 @@
       </c>
       <c r="AQ9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>t</v>
+        <v>d</v>
       </c>
       <c r="AR9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="AS9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>t</v>
       </c>
       <c r="AT9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="AU9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="AV9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>s</v>
       </c>
       <c r="AW9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -23827,27 +23827,27 @@
       </c>
       <c r="AX9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>t</v>
+        <v>d</v>
       </c>
       <c r="AY9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="AZ9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>t</v>
       </c>
       <c r="BA9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="BB9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="BC9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>s</v>
       </c>
       <c r="BD9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -23855,27 +23855,27 @@
       </c>
       <c r="BE9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>t</v>
+        <v>d</v>
       </c>
       <c r="BF9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>s</v>
       </c>
       <c r="BG9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>q</v>
+        <v>t</v>
       </c>
       <c r="BH9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="BI9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>s</v>
+        <v>q</v>
       </c>
       <c r="BJ9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>d</v>
+        <v>s</v>
       </c>
       <c r="BK9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
@@ -23883,7 +23883,7 @@
       </c>
       <c r="BL9" s="88" t="str">
         <f t="shared" ca="1" si="3"/>
-        <v>t</v>
+        <v>d</v>
       </c>
     </row>
     <row r="10" spans="1:68" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
@@ -24203,7 +24203,7 @@
       </c>
       <c r="F12" s="54">
         <f ca="1">TODAY()</f>
-        <v>46189</v>
+        <v>46201</v>
       </c>
       <c r="G12" s="55">
         <v>3</v>
@@ -24446,7 +24446,7 @@
       <c r="E13" s="53"/>
       <c r="F13" s="54">
         <f ca="1">TODAY()+5</f>
-        <v>46194</v>
+        <v>46206</v>
       </c>
       <c r="G13" s="55">
         <v>1</v>
@@ -24691,7 +24691,7 @@
       </c>
       <c r="F14" s="54">
         <f ca="1">F12-3</f>
-        <v>46186</v>
+        <v>46198</v>
       </c>
       <c r="G14" s="55">
         <v>10</v>
@@ -24934,7 +24934,7 @@
       <c r="E15" s="53"/>
       <c r="F15" s="54">
         <f ca="1">F12+20</f>
-        <v>46209</v>
+        <v>46221</v>
       </c>
       <c r="G15" s="55">
         <v>1</v>
@@ -25179,7 +25179,7 @@
       </c>
       <c r="F16" s="54">
         <f ca="1">F12+6</f>
-        <v>46195</v>
+        <v>46207</v>
       </c>
       <c r="G16" s="55">
         <v>6</v>
@@ -25660,7 +25660,7 @@
       </c>
       <c r="F18" s="54">
         <f ca="1">F12+6</f>
-        <v>46195</v>
+        <v>46207</v>
       </c>
       <c r="G18" s="55">
         <v>13</v>
@@ -25905,7 +25905,7 @@
       </c>
       <c r="F19" s="54">
         <f ca="1">F18+2</f>
-        <v>46197</v>
+        <v>46209</v>
       </c>
       <c r="G19" s="55">
         <v>9</v>
@@ -26150,7 +26150,7 @@
       </c>
       <c r="F20" s="54">
         <f ca="1">F19+5</f>
-        <v>46202</v>
+        <v>46214</v>
       </c>
       <c r="G20" s="55">
         <v>11</v>
@@ -26393,7 +26393,7 @@
       <c r="E21" s="53"/>
       <c r="F21" s="54">
         <f ca="1">F20+2</f>
-        <v>46204</v>
+        <v>46216</v>
       </c>
       <c r="G21" s="55">
         <v>1</v>
@@ -26634,7 +26634,7 @@
       <c r="E22" s="53"/>
       <c r="F22" s="54">
         <f ca="1">F21+1</f>
-        <v>46205</v>
+        <v>46217</v>
       </c>
       <c r="G22" s="55">
         <v>24</v>
@@ -27113,7 +27113,7 @@
       <c r="E24" s="53"/>
       <c r="F24" s="54">
         <f ca="1">F12+15</f>
-        <v>46204</v>
+        <v>46216</v>
       </c>
       <c r="G24" s="55">
         <v>4</v>
@@ -27356,7 +27356,7 @@
       <c r="E25" s="53"/>
       <c r="F25" s="54">
         <f ca="1">F24+3</f>
-        <v>46207</v>
+        <v>46219</v>
       </c>
       <c r="G25" s="55">
         <v>14</v>
@@ -27599,7 +27599,7 @@
       <c r="E26" s="53"/>
       <c r="F26" s="54">
         <f ca="1">F25+15</f>
-        <v>46222</v>
+        <v>46234</v>
       </c>
       <c r="G26" s="55">
         <v>6</v>
@@ -27842,7 +27842,7 @@
       <c r="E27" s="53"/>
       <c r="F27" s="54">
         <f ca="1">F21+22</f>
-        <v>46226</v>
+        <v>46238</v>
       </c>
       <c r="G27" s="55">
         <v>3</v>
@@ -28085,7 +28085,7 @@
       <c r="E28" s="53"/>
       <c r="F28" s="54">
         <f ca="1">F16</f>
-        <v>46195</v>
+        <v>46207</v>
       </c>
       <c r="G28" s="55">
         <v>19</v>
@@ -28562,7 +28562,7 @@
       <c r="E30" s="53"/>
       <c r="F30" s="54">
         <f ca="1">F27+3</f>
-        <v>46229</v>
+        <v>46241</v>
       </c>
       <c r="G30" s="55">
         <v>15</v>
@@ -28803,7 +28803,7 @@
       <c r="E31" s="53"/>
       <c r="F31" s="54">
         <f ca="1">F30+14</f>
-        <v>46243</v>
+        <v>46255</v>
       </c>
       <c r="G31" s="55">
         <v>5</v>
@@ -29046,7 +29046,7 @@
       <c r="E32" s="53"/>
       <c r="F32" s="54">
         <f ca="1">F31+42</f>
-        <v>46285</v>
+        <v>46297</v>
       </c>
       <c r="G32" s="55">
         <v>1</v>
@@ -30241,6 +30241,34 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Url xsi:nil="true"/>
+      <Description xsi:nil="true"/>
+    </Image>
+    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
+    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010079F111ED35F8CC479449609E8A0923A6" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="22a266b9fa9a230c5a512669d8b298c3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xmlns:ns3="16c05727-aa75-4e4a-9b5f-8a80a1165891" xmlns:ns4="230e9df3-be65-4c73-a93b-d1236ebd677e" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="eddc33fff6b14141ee5c74a0d29ea6a1" ns1:_="" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -30516,35 +30544,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA4BA2A8-DB97-40F9-8DB6-154C09C7467C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
+    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Url xsi:nil="true"/>
-      <Description xsi:nil="true"/>
-    </Image>
-    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
-    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{39060724-9CA2-4290-8A0C-B53624A594E7}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{75C87518-DD8E-42CD-8DAC-291A323E849B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -30563,24 +30583,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{39060724-9CA2-4290-8A0C-B53624A594E7}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA4BA2A8-DB97-40F9-8DB6-154C09C7467C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
-    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>